<commit_message>
update: get funds name, isin and url
</commit_message>
<xml_diff>
--- a/spreadsheet/interactive_investor.xlsx
+++ b/spreadsheet/interactive_investor.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,13 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,15 +64,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -428,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -459,7 +469,63 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scottish Mortgage </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GB00BLDYK618</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/investment-trusts/scottish-mortgage-ord/LSE:SMT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alliance Witan </t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GB00B11V7W98</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/investment-trusts/alliance-witan-ord/LSE:ALW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">City of London </t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GB0001990497</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/investment-trusts/city-of-london-ord/LSE:CTY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -470,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -501,7 +567,63 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Vanguard S&amp;P 500 UCITS ETF GBP</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>IE00B3XXRP09</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/etfs/vanguard-sp-500-ucits-etf-gbp/LSE:VUSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Vanguard S&amp;P 500 ETF USD Acc GBP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>IE00BFMXXD54</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/etfs/vanguard-sp-500-etf-usd-acc-gbp/LSE:VUAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE All-World ETF USD Acc GBP</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IE00BK5BQT80</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/etfs/vanguard-ftse-all-world-etf-usd-acc-gbp/LSE:VWRP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -512,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -543,7 +665,207 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Vanguard LifeStrategy 80% Equity A Acc</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GB00B4PQW151</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/vanguard-lifestrategy-80-equity-a-acc/B4PQW15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Royal London Short Term Money Mkt Y Acc</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GB00B8XYYQ86</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/royal-london-short-term-money-mkt-y-acc/B8XYYQ8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fundsmith Equity I Acc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GB00B41YBW71</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/fundsmith-equity-i-acc/B41YBW7</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fundsmith Equity R Acc</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GB00B4LPDJ14</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/fundsmith-equity-r-acc/B4LPDJ1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fundsmith Equity T Acc</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GB00B4Q5X527</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/fundsmith-equity-t-acc/B4Q5X52</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Artemis Global Income I Acc</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GB00B5ZX1M70</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/artemis-global-income-i-acc/B5ZX1M7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Artemis Global Income I Inc</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GB00B5N99561</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/artemis-global-income-i-inc/B5N9956</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE UK Eq Inc Idx £ Acc</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GB00B59G4H82</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/vanguard-ftse-uk-eq-inc-idx-acc/B59G4H8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE UK Eq Inc Idx £ Inc</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GB00B5B74684</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/vanguard-ftse-uk-eq-inc-idx-inc/B5B7468</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rathbone M-A Strategic Income Port S Acc</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GB00BY9BT482</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/rathbone-m-a-strategic-income-port-s-acc/BY9BT48</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rathbone M-A Strategic Income Port S Inc</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>GB00BY9BSL83</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ii.co.uk/funds/rathbone-m-a-strategic-income-port-s-inc/BY9BSL8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>